<commit_message>
Styled search chanel button and Header
</commit_message>
<xml_diff>
--- a/Код.xlsx
+++ b/Код.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GrandYT228\Desktop\Voice-ka\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB915911-A046-45C8-B341-143C7D802A87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE98D43-8457-488A-86A4-DAA876966AD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="3300" windowWidth="21600" windowHeight="11505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22920" yWindow="3465" windowWidth="21600" windowHeight="11505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -379,7 +379,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
@@ -501,15 +501,40 @@
       <c r="A4" s="1">
         <v>46064</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
+      <c r="B4" s="2">
+        <f t="shared" ref="B4:B6" si="1">17+21+25</f>
+        <v>63</v>
+      </c>
+      <c r="C4" s="2">
+        <f t="shared" ref="C4:C7" si="2">8+13</f>
+        <v>21</v>
+      </c>
+      <c r="D4" s="2">
+        <f t="shared" ref="D4:D6" si="3">15+29+27+51</f>
+        <v>122</v>
+      </c>
+      <c r="E4" s="2">
+        <f t="shared" ref="E4:E6" si="4">36+37+11</f>
+        <v>84</v>
+      </c>
+      <c r="F4" s="2">
+        <f t="shared" ref="F4:F6" si="5">6+11+5+12+15</f>
+        <v>49</v>
+      </c>
+      <c r="G4" s="2">
+        <f t="shared" ref="G4:G6" si="6">9+114+38+22+19+27+15+9+15+9+9+37+13</f>
+        <v>336</v>
+      </c>
+      <c r="H4" s="2">
+        <f>13</f>
+        <v>13</v>
+      </c>
       <c r="I4" s="2">
         <f t="shared" si="0"/>
+        <v>688</v>
+      </c>
+      <c r="J4">
+        <f t="shared" ref="J4:J67" si="7">I4-I3</f>
         <v>0</v>
       </c>
     </row>
@@ -517,15 +542,40 @@
       <c r="A5" s="1">
         <v>46065</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
+      <c r="B5" s="2">
+        <f t="shared" si="1"/>
+        <v>63</v>
+      </c>
+      <c r="C5" s="2">
+        <f t="shared" si="2"/>
+        <v>21</v>
+      </c>
+      <c r="D5" s="2">
+        <f t="shared" si="3"/>
+        <v>122</v>
+      </c>
+      <c r="E5" s="2">
+        <f t="shared" si="4"/>
+        <v>84</v>
+      </c>
+      <c r="F5" s="2">
+        <f t="shared" si="5"/>
+        <v>49</v>
+      </c>
+      <c r="G5" s="2">
+        <f t="shared" si="6"/>
+        <v>336</v>
+      </c>
+      <c r="H5" s="2">
+        <f>13</f>
+        <v>13</v>
+      </c>
       <c r="I5" s="2">
         <f t="shared" si="0"/>
+        <v>688</v>
+      </c>
+      <c r="J5">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -533,15 +583,40 @@
       <c r="A6" s="1">
         <v>46066</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="B6" s="2">
+        <f t="shared" si="1"/>
+        <v>63</v>
+      </c>
+      <c r="C6" s="2">
+        <f t="shared" si="2"/>
+        <v>21</v>
+      </c>
+      <c r="D6" s="2">
+        <f t="shared" si="3"/>
+        <v>122</v>
+      </c>
+      <c r="E6" s="2">
+        <f t="shared" si="4"/>
+        <v>84</v>
+      </c>
+      <c r="F6" s="2">
+        <f t="shared" si="5"/>
+        <v>49</v>
+      </c>
+      <c r="G6" s="2">
+        <f t="shared" si="6"/>
+        <v>336</v>
+      </c>
+      <c r="H6" s="2">
+        <f>13</f>
+        <v>13</v>
+      </c>
       <c r="I6" s="2">
         <f t="shared" si="0"/>
+        <v>688</v>
+      </c>
+      <c r="J6">
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
@@ -549,16 +624,41 @@
       <c r="A7" s="1">
         <v>46067</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="B7" s="2">
+        <f>23+37+25</f>
+        <v>85</v>
+      </c>
+      <c r="C7" s="2">
+        <f t="shared" si="2"/>
+        <v>21</v>
+      </c>
+      <c r="D7" s="2">
+        <f>46+66+27+15</f>
+        <v>154</v>
+      </c>
+      <c r="E7" s="2">
+        <f>11+36+36+11+11</f>
+        <v>105</v>
+      </c>
+      <c r="F7" s="2">
+        <f>9+13+13+13+6+11+5+12</f>
+        <v>82</v>
+      </c>
+      <c r="G7" s="2">
+        <f>9+110+38+21+20+25+15+8+15+9+9+34+13</f>
+        <v>326</v>
+      </c>
+      <c r="H7" s="2">
+        <f>13</f>
+        <v>13</v>
+      </c>
       <c r="I7" s="2">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>786</v>
+      </c>
+      <c r="J7">
+        <f t="shared" si="7"/>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -576,6 +676,1375 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
+      <c r="J8">
+        <f t="shared" si="7"/>
+        <v>-786</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>46069</v>
+      </c>
+      <c r="I9" s="2">
+        <f t="shared" ref="I9:I72" si="8">SUM(B9:H9)</f>
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>46070</v>
+      </c>
+      <c r="I10" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>46071</v>
+      </c>
+      <c r="I11" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>46072</v>
+      </c>
+      <c r="I12" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>46073</v>
+      </c>
+      <c r="I13" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>46074</v>
+      </c>
+      <c r="I14" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>46075</v>
+      </c>
+      <c r="I15" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>46076</v>
+      </c>
+      <c r="I16" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>46077</v>
+      </c>
+      <c r="I17" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>46078</v>
+      </c>
+      <c r="I18" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>46079</v>
+      </c>
+      <c r="I19" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>46080</v>
+      </c>
+      <c r="I20" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>46081</v>
+      </c>
+      <c r="I21" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>46082</v>
+      </c>
+      <c r="I22" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>46083</v>
+      </c>
+      <c r="I23" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>46084</v>
+      </c>
+      <c r="I24" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>46085</v>
+      </c>
+      <c r="I25" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>46086</v>
+      </c>
+      <c r="I26" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>46087</v>
+      </c>
+      <c r="I27" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>46088</v>
+      </c>
+      <c r="I28" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>46089</v>
+      </c>
+      <c r="I29" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J29">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>46090</v>
+      </c>
+      <c r="I30" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>46091</v>
+      </c>
+      <c r="I31" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>46092</v>
+      </c>
+      <c r="I32" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>46093</v>
+      </c>
+      <c r="I33" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J33">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>46094</v>
+      </c>
+      <c r="I34" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J34">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>46095</v>
+      </c>
+      <c r="I35" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J35">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>46096</v>
+      </c>
+      <c r="I36" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>46097</v>
+      </c>
+      <c r="I37" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>46098</v>
+      </c>
+      <c r="I38" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>46099</v>
+      </c>
+      <c r="I39" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J39">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>46100</v>
+      </c>
+      <c r="I40" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J40">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>46101</v>
+      </c>
+      <c r="I41" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>46102</v>
+      </c>
+      <c r="I42" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J42">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>46103</v>
+      </c>
+      <c r="I43" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J43">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>46104</v>
+      </c>
+      <c r="I44" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J44">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>46105</v>
+      </c>
+      <c r="I45" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J45">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>46106</v>
+      </c>
+      <c r="I46" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J46">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>46107</v>
+      </c>
+      <c r="I47" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J47">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>46108</v>
+      </c>
+      <c r="I48" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J48">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>46109</v>
+      </c>
+      <c r="I49" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J49">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>46110</v>
+      </c>
+      <c r="I50" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J50">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>46111</v>
+      </c>
+      <c r="I51" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J51">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>46112</v>
+      </c>
+      <c r="I52" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J52">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>46113</v>
+      </c>
+      <c r="I53" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J53">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>46114</v>
+      </c>
+      <c r="I54" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J54">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>46115</v>
+      </c>
+      <c r="I55" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J55">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>46116</v>
+      </c>
+      <c r="I56" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J56">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>46117</v>
+      </c>
+      <c r="I57" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J57">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>46118</v>
+      </c>
+      <c r="I58" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J58">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>46119</v>
+      </c>
+      <c r="I59" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J59">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>46120</v>
+      </c>
+      <c r="I60" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J60">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>46121</v>
+      </c>
+      <c r="I61" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J61">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>46122</v>
+      </c>
+      <c r="I62" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J62">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
+        <v>46123</v>
+      </c>
+      <c r="I63" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J63">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>46124</v>
+      </c>
+      <c r="I64" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J64">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>46125</v>
+      </c>
+      <c r="I65" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J65">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
+        <v>46126</v>
+      </c>
+      <c r="I66" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J66">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>46127</v>
+      </c>
+      <c r="I67" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J67">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>46128</v>
+      </c>
+      <c r="I68" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J68">
+        <f t="shared" ref="J68:J113" si="9">I68-I67</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" s="1">
+        <v>46129</v>
+      </c>
+      <c r="I69" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J69">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>46130</v>
+      </c>
+      <c r="I70" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J70">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>46131</v>
+      </c>
+      <c r="I71" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J71">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
+        <v>46132</v>
+      </c>
+      <c r="I72" s="2">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="J72">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A73" s="1">
+        <v>46133</v>
+      </c>
+      <c r="I73" s="2">
+        <f t="shared" ref="I73:I113" si="10">SUM(B73:H73)</f>
+        <v>0</v>
+      </c>
+      <c r="J73">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A74" s="1">
+        <v>46134</v>
+      </c>
+      <c r="I74" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J74">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A75" s="1">
+        <v>46135</v>
+      </c>
+      <c r="I75" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J75">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A76" s="1">
+        <v>46136</v>
+      </c>
+      <c r="I76" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J76">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
+        <v>46137</v>
+      </c>
+      <c r="I77" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J77">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A78" s="1">
+        <v>46138</v>
+      </c>
+      <c r="I78" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J78">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
+        <v>46139</v>
+      </c>
+      <c r="I79" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J79">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
+        <v>46140</v>
+      </c>
+      <c r="I80" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J80">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
+        <v>46141</v>
+      </c>
+      <c r="I81" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J81">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A82" s="1">
+        <v>46142</v>
+      </c>
+      <c r="I82" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J82">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A83" s="1">
+        <v>46143</v>
+      </c>
+      <c r="I83" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J83">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A84" s="1">
+        <v>46144</v>
+      </c>
+      <c r="I84" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J84">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A85" s="1">
+        <v>46145</v>
+      </c>
+      <c r="I85" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J85">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A86" s="1">
+        <v>46146</v>
+      </c>
+      <c r="I86" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J86">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A87" s="1">
+        <v>46147</v>
+      </c>
+      <c r="I87" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J87">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A88" s="1">
+        <v>46148</v>
+      </c>
+      <c r="I88" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J88">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A89" s="1">
+        <v>46149</v>
+      </c>
+      <c r="I89" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J89">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A90" s="1">
+        <v>46150</v>
+      </c>
+      <c r="I90" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J90">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A91" s="1">
+        <v>46151</v>
+      </c>
+      <c r="I91" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J91">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A92" s="1">
+        <v>46152</v>
+      </c>
+      <c r="I92" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J92">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A93" s="1">
+        <v>46153</v>
+      </c>
+      <c r="I93" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J93">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A94" s="1">
+        <v>46154</v>
+      </c>
+      <c r="I94" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J94">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A95" s="1">
+        <v>46155</v>
+      </c>
+      <c r="I95" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J95">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A96" s="1">
+        <v>46156</v>
+      </c>
+      <c r="I96" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J96">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A97" s="1">
+        <v>46157</v>
+      </c>
+      <c r="I97" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J97">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A98" s="1">
+        <v>46158</v>
+      </c>
+      <c r="I98" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J98">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A99" s="1">
+        <v>46159</v>
+      </c>
+      <c r="I99" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J99">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A100" s="1">
+        <v>46160</v>
+      </c>
+      <c r="I100" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J100">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A101" s="1">
+        <v>46161</v>
+      </c>
+      <c r="I101" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J101">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A102" s="1">
+        <v>46162</v>
+      </c>
+      <c r="I102" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J102">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A103" s="1">
+        <v>46163</v>
+      </c>
+      <c r="I103" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J103">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A104" s="1">
+        <v>46164</v>
+      </c>
+      <c r="I104" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J104">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A105" s="1">
+        <v>46165</v>
+      </c>
+      <c r="I105" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J105">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A106" s="1">
+        <v>46166</v>
+      </c>
+      <c r="I106" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J106">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A107" s="1">
+        <v>46167</v>
+      </c>
+      <c r="I107" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J107">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A108" s="1">
+        <v>46168</v>
+      </c>
+      <c r="I108" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J108">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A109" s="1">
+        <v>46169</v>
+      </c>
+      <c r="I109" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J109">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A110" s="1">
+        <v>46170</v>
+      </c>
+      <c r="I110" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J110">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A111" s="1">
+        <v>46171</v>
+      </c>
+      <c r="I111" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J111">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A112" s="1">
+        <v>46172</v>
+      </c>
+      <c r="I112" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J112">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A113" s="1">
+        <v>46173</v>
+      </c>
+      <c r="I113" s="2">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="J113">
+        <f t="shared" si="9"/>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>